<commit_message>
sync: actualizar bases de datos de remisiones y corte/doblez en sync_databases para Streamlit Cloud
</commit_message>
<xml_diff>
--- a/data/sync_databases/BD_Actividad_Log.xlsx
+++ b/data/sync_databases/BD_Actividad_Log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J646"/>
+  <dimension ref="A1:J699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28864,6 +28864,2338 @@
         </is>
       </c>
     </row>
+    <row r="647">
+      <c r="A647" t="n">
+        <v>646</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>18:40:32</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0511 cargada con 264 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>TPM-0511</t>
+        </is>
+      </c>
+      <c r="H647" t="n">
+        <v>264</v>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>PO 2608-3177</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" t="n">
+        <v>647</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>21:16:14</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Remisión E0126 generada con 3 tarima(s) y 368 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>E0126</t>
+        </is>
+      </c>
+      <c r="H648" t="n">
+        <v>368</v>
+      </c>
+      <c r="I648" t="inlineStr"/>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>648</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>21:16:16</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0513 marcada como Remesada en E0126 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>TPM-0513</t>
+        </is>
+      </c>
+      <c r="H649" t="n">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr"/>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>649</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>21:16:18</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0512 marcada como Remesada en E0126 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>TPM-0512</t>
+        </is>
+      </c>
+      <c r="H650" t="n">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr"/>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>650</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>21:16:20</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0511 marcada como Remesada en E0126 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>TPM-0511</t>
+        </is>
+      </c>
+      <c r="H651" t="n">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr"/>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>651</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>23:12:33</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Remisión E0126 generada con 3 tarima(s) y 368 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>E0126</t>
+        </is>
+      </c>
+      <c r="H652" t="n">
+        <v>368</v>
+      </c>
+      <c r="I652" t="inlineStr"/>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>652</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>15:10:38</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Remisión E0127 generada con 6 tarima(s) y 190 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>E0127</t>
+        </is>
+      </c>
+      <c r="H653" t="n">
+        <v>190</v>
+      </c>
+      <c r="I653" t="inlineStr"/>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>653</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>15:10:41</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0236 marcada como Remesada en E0127 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>TPM-0236</t>
+        </is>
+      </c>
+      <c r="H654" t="n">
+        <v>0</v>
+      </c>
+      <c r="I654" t="inlineStr"/>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>654</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>15:10:42</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0238 marcada como Remesada en E0127 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>TPM-0238</t>
+        </is>
+      </c>
+      <c r="H655" t="n">
+        <v>0</v>
+      </c>
+      <c r="I655" t="inlineStr"/>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>655</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>15:48:38</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Remisión E0128 generada con 6 tarima(s) y 175 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>E0128</t>
+        </is>
+      </c>
+      <c r="H656" t="n">
+        <v>175</v>
+      </c>
+      <c r="I656" t="inlineStr"/>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>656</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>15:48:40</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0499 marcada como Remesada en E0128 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>TPM-0499</t>
+        </is>
+      </c>
+      <c r="H657" t="n">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr"/>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>657</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>17:44:20</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0514 cargada con 60 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>TPM-0514</t>
+        </is>
+      </c>
+      <c r="H658" t="n">
+        <v>60</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" t="n">
+        <v>658</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>17:45:19</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Remisión E0129 generada con 1 tarima(s) y 60 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>E0129</t>
+        </is>
+      </c>
+      <c r="H659" t="n">
+        <v>60</v>
+      </c>
+      <c r="I659" t="inlineStr"/>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>659</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>17:45:21</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0514 marcada como Remesada en E0129 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>TPM-0514</t>
+        </is>
+      </c>
+      <c r="H660" t="n">
+        <v>0</v>
+      </c>
+      <c r="I660" t="inlineStr"/>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="n">
+        <v>660</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>23:37:06</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0515 cargada con 404 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="H661" t="n">
+        <v>404</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr"/>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>661</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>19:05:47</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0516 cargada con 144 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>TPM-0516</t>
+        </is>
+      </c>
+      <c r="H662" t="n">
+        <v>144</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr"/>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>662</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>20:47:47</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0518 cargada con 8 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>TPM-0518</t>
+        </is>
+      </c>
+      <c r="H663" t="n">
+        <v>8</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" t="n">
+        <v>663</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>20:51:09</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0518 cargada con 8 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>TPM-0518</t>
+        </is>
+      </c>
+      <c r="H664" t="n">
+        <v>8</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" t="n">
+        <v>664</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>20:51:12</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0519 cargada con 128 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>TPM-0519</t>
+        </is>
+      </c>
+      <c r="H665" t="n">
+        <v>128</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" t="n">
+        <v>665</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Remisión E0130 generada con 7 tarima(s) y 860 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>E0130</t>
+        </is>
+      </c>
+      <c r="H666" t="n">
+        <v>860</v>
+      </c>
+      <c r="I666" t="inlineStr"/>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="n">
+        <v>666</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>15:35:21</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Remisión E0131 generada con 6 tarima(s) y 157 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>E0131</t>
+        </is>
+      </c>
+      <c r="H667" t="n">
+        <v>157</v>
+      </c>
+      <c r="I667" t="inlineStr"/>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="n">
+        <v>667</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>15:35:23</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0276 marcada como Remesada en E0131 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>TPM-0276</t>
+        </is>
+      </c>
+      <c r="H668" t="n">
+        <v>0</v>
+      </c>
+      <c r="I668" t="inlineStr"/>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="n">
+        <v>668</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>15:35:26</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0502 marcada como Remesada en E0131 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>TPM-0502</t>
+        </is>
+      </c>
+      <c r="H669" t="n">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr"/>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="n">
+        <v>669</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>21:22:31</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0522 cargada con 211 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>TPM-0522</t>
+        </is>
+      </c>
+      <c r="H670" t="n">
+        <v>211</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>PO 2608-3382; PO 2608-3428; PO 2608-3394</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr"/>
+    </row>
+    <row r="671">
+      <c r="A671" t="n">
+        <v>670</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>21:41:47</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Remisión E0132 generada con 6 tarima(s) y 309 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>E0132</t>
+        </is>
+      </c>
+      <c r="H671" t="n">
+        <v>309</v>
+      </c>
+      <c r="I671" t="inlineStr"/>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="n">
+        <v>671</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>21:41:51</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0456 marcada como Remesada en E0132 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>TPM-0456</t>
+        </is>
+      </c>
+      <c r="H672" t="n">
+        <v>0</v>
+      </c>
+      <c r="I672" t="inlineStr"/>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="n">
+        <v>672</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>21:41:58</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0444 marcada como Remesada en E0132 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>TPM-0444</t>
+        </is>
+      </c>
+      <c r="H673" t="n">
+        <v>0</v>
+      </c>
+      <c r="I673" t="inlineStr"/>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="n">
+        <v>673</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>21:42:05</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0326 marcada como Remesada en E0132 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>TPM-0326</t>
+        </is>
+      </c>
+      <c r="H674" t="n">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr"/>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="n">
+        <v>674</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>21:42:07</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0500 marcada como Remesada en E0132 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>TPM-0500</t>
+        </is>
+      </c>
+      <c r="H675" t="n">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr"/>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="n">
+        <v>675</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>21:45:57</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Remisión E0133 generada con 1 tarima(s) y 1 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>E0133</t>
+        </is>
+      </c>
+      <c r="H676" t="n">
+        <v>1</v>
+      </c>
+      <c r="I676" t="inlineStr"/>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="n">
+        <v>676</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>14:23:12</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0524 cargada con 233 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>TPM-0524</t>
+        </is>
+      </c>
+      <c r="H677" t="n">
+        <v>233</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="n">
+        <v>677</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>14:23:14</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0525 cargada con 123 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>TPM-0525</t>
+        </is>
+      </c>
+      <c r="H678" t="n">
+        <v>123</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="n">
+        <v>678</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>15:10:45</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0527 cargada con 26 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>TPM-0527</t>
+        </is>
+      </c>
+      <c r="H679" t="n">
+        <v>26</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="n">
+        <v>679</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>15:10:46</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0528 cargada con 30 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>TPM-0528</t>
+        </is>
+      </c>
+      <c r="H680" t="n">
+        <v>30</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="n">
+        <v>680</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>15:10:48</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0529 cargada con 30 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>TPM-0529</t>
+        </is>
+      </c>
+      <c r="H681" t="n">
+        <v>30</v>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="n">
+        <v>681</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>15:10:50</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0530 cargada con 18 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>TPM-0530</t>
+        </is>
+      </c>
+      <c r="H682" t="n">
+        <v>18</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="n">
+        <v>682</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>15:10:52</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0531 cargada con 12 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>TPM-0531</t>
+        </is>
+      </c>
+      <c r="H683" t="n">
+        <v>12</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" t="n">
+        <v>683</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>15:10:55</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0532 cargada con 30 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>TPM-0532</t>
+        </is>
+      </c>
+      <c r="H684" t="n">
+        <v>30</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="n">
+        <v>684</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>15:10:57</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0533 cargada con 19 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>TPM-0533</t>
+        </is>
+      </c>
+      <c r="H685" t="n">
+        <v>19</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="n">
+        <v>685</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>15:11:00</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0534 cargada con 25 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>TPM-0534</t>
+        </is>
+      </c>
+      <c r="H686" t="n">
+        <v>25</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="n">
+        <v>686</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>16:07:02</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0539 cargada con 22 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>TPM-0539</t>
+        </is>
+      </c>
+      <c r="H687" t="n">
+        <v>22</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr"/>
+    </row>
+    <row r="688">
+      <c r="A688" t="n">
+        <v>687</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>16:07:05</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0540 cargada con 26 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>TPM-0540</t>
+        </is>
+      </c>
+      <c r="H688" t="n">
+        <v>26</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="n">
+        <v>688</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>16:56:03</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Remisión E0134 generada con 5 tarima(s) y 936 piezas hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>E0134</t>
+        </is>
+      </c>
+      <c r="H689" t="n">
+        <v>936</v>
+      </c>
+      <c r="I689" t="inlineStr"/>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="n">
+        <v>689</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>16:56:05</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0524 marcada como Remesada en E0134 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>TPM-0524</t>
+        </is>
+      </c>
+      <c r="H690" t="n">
+        <v>0</v>
+      </c>
+      <c r="I690" t="inlineStr"/>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="n">
+        <v>690</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>16:56:07</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0539 marcada como Remesada en E0134 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>TPM-0539</t>
+        </is>
+      </c>
+      <c r="H691" t="n">
+        <v>0</v>
+      </c>
+      <c r="I691" t="inlineStr"/>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="n">
+        <v>691</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>16:56:09</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0525 marcada como Remesada en E0134 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>TPM-0525</t>
+        </is>
+      </c>
+      <c r="H692" t="n">
+        <v>0</v>
+      </c>
+      <c r="I692" t="inlineStr"/>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="n">
+        <v>692</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>16:56:12</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0526 marcada como Remesada en E0134 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>TPM-0526</t>
+        </is>
+      </c>
+      <c r="H693" t="n">
+        <v>0</v>
+      </c>
+      <c r="I693" t="inlineStr"/>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="n">
+        <v>693</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>16:56:14</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0540 marcada como Remesada en E0134 hacia PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>TPM-0540</t>
+        </is>
+      </c>
+      <c r="H694" t="n">
+        <v>0</v>
+      </c>
+      <c r="I694" t="inlineStr"/>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="n">
+        <v>694</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>21:43:13</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0541 cargada con 28 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>TPM-0541</t>
+        </is>
+      </c>
+      <c r="H695" t="n">
+        <v>28</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>PNC</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="n">
+        <v>695</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>15:46:09</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0542 cargada con 11 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>TPM-0542</t>
+        </is>
+      </c>
+      <c r="H696" t="n">
+        <v>11</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>PO 2608-3494; PO 2608-3486; PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="n">
+        <v>696</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>17:11:27</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>REMISION_NUEVA</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Remisión E0135 generada con 6 tarima(s) y 97 piezas hacia EQM</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>E0135</t>
+        </is>
+      </c>
+      <c r="H697" t="n">
+        <v>97</v>
+      </c>
+      <c r="I697" t="inlineStr"/>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="n">
+        <v>697</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>17:11:29</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>TARIMA_REMESADA</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Tarima TPM-0547 marcada como Remesada en E0135 hacia EQM</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>TPM-0547</t>
+        </is>
+      </c>
+      <c r="H698" t="n">
+        <v>0</v>
+      </c>
+      <c r="I698" t="inlineStr"/>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="n">
+        <v>698</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>18:28:53</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>TARIMA_NUEVA</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Nueva tarima TPM-0548 cargada con 14 piezas (Cuadrada)</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>TPM-0548</t>
+        </is>
+      </c>
+      <c r="H699" t="n">
+        <v>14</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>PO 2602-0711</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>